<commit_message>
Show CO Perfect Store PDP media
</commit_message>
<xml_diff>
--- a/base_prov_co/cruz_verde/cruz_verde_abbott_2026_09_22.xlsx
+++ b/base_prov_co/cruz_verde/cruz_verde_abbott_2026_09_22.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:Q50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,10 +496,20 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>url_imagen</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>url_producto</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>disponibilidad</t>
         </is>
@@ -556,13 +566,25 @@
       <c r="L2" t="n">
         <v>53</v>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>135</v>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Encuentra Ensure Advance 850 g en Cruz Verde. Úsalo como apoyo nutricional o de bienestar según indicación, formato y datos del envase.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwa7ad7a7a/images/large/129816_5Ensure_Advance_Vainilla_Con_Proteina___HMB_Polvo_850g.jpg</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-vainilla-con-proteina--hmb-polvo-850g/COCV_129816.html</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -619,13 +641,25 @@
       <c r="L3" t="n">
         <v>46</v>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>148</v>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>Ensure Advance Lata x 850 g + Lata x 400 g disponible en Cruz Verde para rutinas de nutrición y bienestar. Compra online y confirma su presentación.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwcd1d9ad1/images/large/163576_1_Promo_Ensure_Advance_Lata_x_850g_Lata_x_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/promo-ensure-advance-lata-x-850g--lata-x-400g/COCV_163576.html</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -682,13 +716,25 @@
       <c r="L4" t="n">
         <v>57</v>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>213</v>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>Ensure® Advance contiene HMB, proteína y 28 vitaminas y minerales incluyendo calcio y vitamina D. Ayuda a recuperar la masa muscular perdida por una condición de salud, y a mejorar la vitalidad, fuerza y movilidad</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw60dab794/images/large/402006_5Ensure_Advance_Vainilla_Con_Proteina___HMB_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-vainilla-liquido-220-ml/COCV_402006.html</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -745,13 +791,25 @@
       <c r="L5" t="n">
         <v>71</v>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>145</v>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>Encuentra Promo Ensure Advance Vainilla en Cruz Verde. Considera presentación, contenido, formato y recomendaciones del empaque antes de comprar.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw9556e8f3/images/large/547197_1_PROMO_ENSURE_ADVANCE_PREC_ESP_CAJ_X_6FCOS_X_220ML_VAINILLA.jpg</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-vainilla-con-proteina-liquido-220-ml-caja-por-6-unidades/COCV_547197.html</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -808,13 +866,25 @@
       <c r="L6" t="n">
         <v>53</v>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>153</v>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>Ensure Advance Vainilla en Cruz Verde: considera presentación, sabor, formato, etapa y recomendaciones del empaque antes de comprar según disponibilidad.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw033080f8/images/large/111380_5Ensure_Advance_Vainilla_Con_Proteina___HMB_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-vainilla-con-proteina--hmb-polvo-400g/COCV_111380.html</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -871,13 +941,25 @@
       <c r="L7" t="n">
         <v>57</v>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>125</v>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>Ensure Advance sabor fresa en formato líquido de 220 ml. Revisa contenido, porción e información nutricional antes de elegir.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwcaced56c/images/large/402008_5Ensure_Advance_Fresa_Con_Proteina___HMB_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-fresa-con-proteina--hmb-liquido-220-ml/COCV_402008.html</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -934,13 +1016,25 @@
       <c r="L8" t="n">
         <v>50</v>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>136</v>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
+          <t>Compra Ensure Fresa 850 g online en Cruz Verde. Considera formato, sabor y porción sugerida según la presentación del producto en línea.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw8ca46b74/images/large/163112_5Ensure_Advance_Fresa_Con_Proteina___HMB_Polvo_850g.jpg</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-fresa-con-proteina--hmb-polvo-850g/COCV_163112.html</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -997,13 +1091,25 @@
       <c r="L9" t="n">
         <v>50</v>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>213</v>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
+          <t>Ensure® Advance contiene HMB, proteína y 28 vitaminas y minerales incluyendo calcio y vitamina D. Ayuda a recuperar la masa muscular perdida por una condición de salud, y a mejorar la vitalidad, fuerza y movilidad</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw99cdb483/images/large/163111_3_Ensure_Advance_Fresa_Con_Proteina___HMB_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-fresa-polvo-400-gr/COCV_163111.html</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1060,13 +1166,25 @@
       <c r="L10" t="n">
         <v>58</v>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>146</v>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
+          <t>Ensure Advance Chocolate Liquido 220 ml en Cruz Verde: considera formato, porción sugerida y recomendaciones del fabricante antes de incorporarlo.</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwe3c35804/images/large/402007_5Ensure_Advance_Chocolate_Con_Proteina___HMB_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-chocolate-con-proteina--hmb-liquido-220-ml/COCV_402007.html</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1123,13 +1241,25 @@
       <c r="L11" t="n">
         <v>31</v>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>143</v>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
+          <t>Ensure Vainilla Polvo 400 g en Cruz Verde: considera presentación, sabor, cantidad y orientación profesional antes de incorporarlo a tu rutina.</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw311c3983/images/large/109254_5Ensure_Base_Vainilla_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-base-vainilla-polvo-400g/COCV_109254.html</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1186,13 +1316,25 @@
       <c r="L12" t="n">
         <v>35</v>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>138</v>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
+          <t>Un vaso de Ensure® proporciona: 28 vitaminas y minerales esenciales, calcio y antioxidantes, vitamina D, omega-3 y es fuente de fibra FOS.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwd7b95be5/images/large/532007_5Ensure_Base_Vainilla_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-vainilla-liquido-220-ml/COCV_532007.html</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1249,13 +1391,25 @@
       <c r="L13" t="n">
         <v>53</v>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>230</v>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
+          <t>Ensure® Advance es nutrición especializada para adultos con HMB, proteína y 28 vitaminas y minerales. Ideal para ayudar a recuperar la masa muscular perdida por una condición de salud, y a mejorar la vitalidad, fuerza y movilidad.</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwfc33ec59/images/large/530022_5Ensure_Advance_Cafe_Con_Proteina___HMB_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-cafe-liquido-220-ml/COCV_530022.html</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1312,13 +1466,25 @@
       <c r="L14" t="n">
         <v>49</v>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>55</v>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
+          <t>Ensure Advance Nutricion Especializada Tarro 400Gr Cafe</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw2b5231fd/images/large/578454_5Ensure_Advance_Cafe_Con_Proteina___HMB_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/ensure-advance-nutricion-especializada-tarro-400gr-cafe/COCV_578454.html</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1375,13 +1541,25 @@
       <c r="L15" t="n">
         <v>50</v>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>136</v>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
+          <t>Glucerna 850 Gr 850 g disponible en Cruz Verde para rutinas de nutrición y bienestar. Compra online y confirma su presentación en línea.</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw7dd3d0c2/images/large/577824_5Glucerna_Formula_para_Diabetes_Polvo_Vainilla_850g.jpg</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/glucerna-tarro-x-850gr-vainilla/COCV_577824.html</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1438,13 +1616,25 @@
       <c r="L16" t="n">
         <v>54</v>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>222</v>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
+          <t>¡Controla tus niveles de azúcar! Glucerna® te ayuda a estabilizar tus niveles de azúcar desde el primer día gracias a su doble método de acción que permite mejorar la producción de insulina y reducir la resistencia a ella.</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwa7746763/images/large/128687_5Glucerna_Forrmula_para_Diabetes_Liquido_Vainilla_237_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/glucerna-vainilla-liquido-220-ml/COCV_128687.html</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1501,13 +1691,25 @@
       <c r="L17" t="n">
         <v>82</v>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>138</v>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
+          <t>Compra Glucerna por 1 Tarro por 850gr+ 1 400gr Vainilla online en Cruz Verde. Considera formato, sabor y porción sugerida antes de usarlo.</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw056bc6e5/images/large/572641_1_Promo_Glucerna_Descuento_Paquete_por_1_Tarro_por_850Gr_1_Tarro_por_400Gr_Vainilla.jpg</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/promo-glucerna-descuento-paquete-por-1-tarro-por-850gr-1-tarro-por-400gr-vainilla/COCV_572641.html</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1564,13 +1766,25 @@
       <c r="L18" t="n">
         <v>52</v>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>155</v>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
+          <t>Glucerna Vainilla Liquido 220 ml en Cruz Verde: considera presentación, disponibilidad, información del empaque y orientación profesional antes de comprar.</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw21866391/images/large/547912_1_PROMO_GLUCERNA_ABBOTT_PREC_ESPE_093KCAL_ML_CAJ_X_6BOT_X_237ML_VAINILLA.jpg</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/glucerna-vainilla-liquido-220-ml-caja-x6-unidades/COCV_547912.html</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1627,13 +1841,25 @@
       <c r="L19" t="n">
         <v>51</v>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>222</v>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
+          <t>¡Controla tus niveles de azúcar! Glucerna® te ayuda a estabilizar tus niveles de azúcar desde el primer día gracias a su doble método de acción que permite mejorar la producción de insulina y reducir la resistencia a ella.</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwa4a7b4c4/images/large/138288_3Glucerna_Formula_para_Diabetes_Liquido_Fresa_237_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/glucerna-fresa-liquido-220-ml/COCV_138288.html</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1690,13 +1916,25 @@
       <c r="L20" t="n">
         <v>50</v>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>154</v>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
+          <t>Glucerna Vainilla Polvo 400 g en Cruz Verde: considera presentación, formato, disponibilidad y datos del empaque antes de elegirlo. según tus necesidades.</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwd8a58e21/images/large/142214_5Glucerna_Formula_para_Diabetes_Polvo_Vainilla_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/glucerna-vainilla-polvo-400-gr/COCV_142214.html</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1753,13 +1991,25 @@
       <c r="L21" t="n">
         <v>24</v>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>105</v>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
+          <t>Referencia: 157457Registro Sanitario: RSA-0035011-2024Incluye 0% de impuestosPresentación: tarro x 400 gr</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>https://copservir.vtexassets.com/arquivos/ids/1942555/GLUCERNA-CAPUCHINO-POLVO_F.png?v=639167595673670000</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
           <t>https://www.larebajavirtual.com/glucerna-capuchino-polvo-157457/p</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1816,13 +2066,25 @@
       <c r="L22" t="n">
         <v>46</v>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>147</v>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
+          <t>Compra Pedialyte Max 60 Uva 500 ml en Cruz Verde. Ten presente formato, presentación, disponibilidad e información del empaque antes de adquirirlo.</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwdcff4817/images/large/96738_1_PEDIALYTE_CON_ZINC_60MEQNa_L_SOL_ORAL_FCO_X_500ML_UVA.jpg</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-max-60-uva-500-ml/COCV_96738.html</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1879,13 +2141,25 @@
       <c r="L23" t="n">
         <v>61</v>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>139</v>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
+          <t>Pedialyte Max 60 sabor fresa de 500 ml, una presentación de suero pediátrico. Revisa concentración, sabor y disponibilidad antes de elegir.</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw40d23db8/images/large/165575_1_PEDIALYTE_MAX_CON_ZINC_60MEQNA_L_SOL_ORAL_FCO_X_500ML_FRESA.jpg</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-max-60-fresa-500-ml/COCV_165575.html</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -1942,13 +2216,25 @@
       <c r="L24" t="n">
         <v>57</v>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>115</v>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
+          <t>Pedialyte Max 60 sabor manzana de 500 ml. Revisa esta presentación de suero oral 60 mEq, su sabor y disponibilidad.</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw76a0427e/images/large/96736_1_PEDIALYTE_CON_ZINC_60MEQNa_L_SOL_ORAL_FCO_X_500ML_MANZANA.jpg</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-max-60-manzana-500-ml/COCV_96736.html</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2005,13 +2291,25 @@
       <c r="L25" t="n">
         <v>47</v>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>151</v>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
+          <t>Suero De Rehidratacion Pedialyte Max 60 Coco 500 ml en Cruz Verde: considera formato, cantidad y condiciones indicadas en el empaque antes de elegirlo.</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwb30e022c/images/large/165574_1_PEDIALYTE_MAX_CON_ZINC_60MEQNA_L_SOL_ORAL_FCO_X_500ML_COCO.jpg</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-max-60-coco-500-ml/COCV_165574.html</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2068,13 +2366,25 @@
       <c r="L26" t="n">
         <v>52</v>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>246</v>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
+          <t>Pedialyte® 30 mEq - 45 mEq está científicamente diseñado para prevenir la deshidratación leve y para hidratar de forma más rápida y efectiva, principalmente en casos de deshidratación por actividad física intensa o exposición prolongada al calor.</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwefb18bd5/images/large/134768_1_PEDIALYTE_CON_ZINC_30MEQNa_L_SOL_ORAL_FCO_X_500ML_CEREZA.jpg</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-active-30-cereza-500-ml/COCV_134768.html</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2131,13 +2441,25 @@
       <c r="L27" t="n">
         <v>51</v>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>246</v>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
+          <t>Pedialyte® 30 mEq - 45 mEq está científicamente diseñado para prevenir la deshidratación leve y para hidratar de forma más rápida y efectiva, principalmente en casos de deshidratación por actividad física intensa o exposición prolongada al calor.</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwe2614e2a/images/large/96734_1_PEDIALYTE_CON_ZINC_45MEQNa_L_SOL_ORAL_FCO_X_500ML_FRESA.jpg</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-active-45-fresa-500-ml/COCV_96734.html</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2194,13 +2516,25 @@
       <c r="L28" t="n">
         <v>50</v>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>246</v>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
+          <t>Pedialyte® 30 mEq - 45 mEq está científicamente diseñado para prevenir la deshidratación leve y para hidratar de forma más rápida y efectiva, principalmente en casos de deshidratación por actividad física intensa o exposición prolongada al calor.</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw23f80837/images/large/134770_1_PEDIALYTE_CON_ZINC_30MEQNa_L_SOL_ORAL_FCO_X_500ML_COCO.jpg</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-active-30-coco-500-ml/COCV_134770.html</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2257,13 +2591,25 @@
       <c r="L29" t="n">
         <v>53</v>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>246</v>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
+          <t>Pedialyte® 30 mEq - 45 mEq está científicamente diseñado para prevenir la deshidratación leve y para hidratar de forma más rápida y efectiva, principalmente en casos de deshidratación por actividad física intensa o exposición prolongada al calor.</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw4053f574/images/large/134769_1_PEDIALYTE_CON_ZINC_30MEQNa_L_SOL_ORAL_FCO_X_500ML_MANZANA.jpg</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-active-30-manzana-500-ml/COCV_134769.html</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2320,13 +2666,25 @@
       <c r="L30" t="n">
         <v>53</v>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>246</v>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
+          <t>Pedialyte® 30 mEq - 45 mEq está científicamente diseñado para prevenir la deshidratación leve y para hidratar de forma más rápida y efectiva, principalmente en casos de deshidratación por actividad física intensa o exposición prolongada al calor.</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwef87bc86/images/large/134771_1_PEDIALYTE_CON_ZINC_30MEQNa_L_SOL_ORAL_FCO_X_500ML_DURAZNO.jpg</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-active-30-durazno-500-ml/COCV_134771.html</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2383,13 +2741,25 @@
       <c r="L31" t="n">
         <v>53</v>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>246</v>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
+          <t>Pedialyte® 30 mEq - 45 mEq está científicamente diseñado para prevenir la deshidratación leve y para hidratar de forma más rápida y efectiva, principalmente en casos de deshidratación por actividad física intensa o exposición prolongada al calor.</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw63e62bd0/images/large/394640_1_PEDIALYTE_ACTIVE_45MEQNa_L_SOL_ORAL_FCO_X_500ML_GUARANA.jpg</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/suero-de-rehidratacion-pedialyte-active-45-guarana-500-ml/COCV_394640.html</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2446,13 +2816,25 @@
       <c r="L32" t="n">
         <v>52</v>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>40</v>
+      </c>
       <c r="N32" t="inlineStr">
         <is>
+          <t>Pediasure Peptigro Tarro por 400Gr Fresa</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwb195808b/images/large/574284_4Pediasure_Formula_Nutricional_Fresa_Ninos_2_10_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-peptigro-tarro-por-400gr-fresa/COCV_574284.html</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="Q32" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2509,13 +2891,25 @@
       <c r="L33" t="n">
         <v>56</v>
       </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>139</v>
+      </c>
       <c r="N33" t="inlineStr">
         <is>
+          <t>Compra PediaSure 1600 1600 g online en Cruz Verde. Considera formato, sabor y porción sugerida según la presentación del producto en línea.</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwc68020e2/images/large/556914_5Pediasure_Formula_Nutricional_Vainilla_Ninos_2_10_liquido_1600g.jpg</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-10kcalml-lata-x-1600gr-vainilla/COCV_556914.html</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="Q33" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2572,13 +2966,25 @@
       <c r="L34" t="n">
         <v>55</v>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>156</v>
+      </c>
       <c r="N34" t="inlineStr">
         <is>
+          <t>Para que tu hijo crezca es importante una adecuada alimentación, apóyalo con Pediasure® y su fórmula especializada, ¡ayúdalo a alcanzar su máximo potencial!</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw3f32c42e/images/large/574305_5Pediasure_Formula_Nutricional_Vainilla_Ninos_2_10_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-peptigro-tarro-por-400gr-vainilla/COCV_574305.html</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2635,13 +3041,25 @@
       <c r="L35" t="n">
         <v>59</v>
       </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>67</v>
+      </c>
       <c r="N35" t="inlineStr">
         <is>
+          <t>Pediasure Vainilla para bienestar diario. Disponible en Cruz Verde.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw511f56fc/images/large/525504_5Pediasure_Formula_Nutricional_Vainilla_Ninos_2_10_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-vainilla-liquido-220ml/COCV_525504.html</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2698,13 +3116,25 @@
       <c r="L36" t="n">
         <v>56</v>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>156</v>
+      </c>
       <c r="N36" t="inlineStr">
         <is>
+          <t>Para que tu hijo crezca es importante una adecuada alimentación, apóyalo con Pediasure® y su fórmula especializada, ¡ayúdalo a alcanzar su máximo potencial!</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwb4d2a900/images/large/525503_5Pediasure_Formula_Nutricional_Fresa_Ninos_2_10_Liquido_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-fresa-liquido-220-ml/COCV_525503.html</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2761,13 +3191,25 @@
       <c r="L37" t="n">
         <v>52</v>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>149</v>
+      </c>
       <c r="N37" t="inlineStr">
         <is>
+          <t>Pediasure Peptigro Tarro por 850 g Fresa en Cruz Verde: considera presentación, sabor, formato, etapa y recomendaciones del empaque antes de comprar.</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw7d9ce4d3/images/large/574283_5Pediasure_Formula_Nutricional_Fresa_Ninos_2_10_Polvo_850g.jpg</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-peptigro-tarro-por-850gr-fresa/COCV_574283.html</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2824,13 +3266,25 @@
       <c r="L38" t="n">
         <v>52</v>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>40</v>
+      </c>
       <c r="N38" t="inlineStr">
         <is>
+          <t>Pediasure Peptigro Tarro por 400Gr Fresa</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwb195808b/images/large/574284_4Pediasure_Formula_Nutricional_Fresa_Ninos_2_10_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-peptigro-tarro-por-400gr-fresa/COCV_574284.html</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="Q38" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2887,13 +3341,25 @@
       <c r="L39" t="n">
         <v>65</v>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>156</v>
+      </c>
       <c r="N39" t="inlineStr">
         <is>
+          <t>Para que tu hijo crezca es importante una adecuada alimentación, apóyalo con Pediasure® y su fórmula especializada, ¡ayúdalo a alcanzar su máximo potencial!</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwf0f87e56/images/large/547911_1PROMO_PEDIASURE_ABBOTT_PREC_ESPE_1.0_KCAL_ML_CAJ_X_6BOT_X_220ML_VAINILLA.jpg</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/promo-pediasure-abbott-precio-especial-10-kcal-ml-caja-x-6bot-x-220ml-vainilla/COCV_547911.html</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -2950,13 +3416,25 @@
       <c r="L40" t="n">
         <v>71</v>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>64</v>
+      </c>
       <c r="N40" t="inlineStr">
         <is>
+          <t>Pediasure Nutricion Especializada 10+ Años Frasco 220Ml Vainilla</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwe7f28b28/images/large/578455_4Pediasure_Formula_Nutricional_para_Adolescentes_10__Vainilla_Polvo_220_Ml.jpg</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/pediasure-nutricion-especializada-10-anos-frasco-220ml-vainilla/COCV_578455.html</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="Q40" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3013,13 +3491,25 @@
       <c r="L41" t="n">
         <v>33</v>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>137</v>
+      </c>
       <c r="N41" t="inlineStr">
         <is>
+          <t>Encuentra Similac Etapa 1 1400 g en Cruz Verde. Úsalo como apoyo nutricional o de bienestar según indicación, formato y datos del envase.</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw098060a4/images/large/547206_3Fomula_Infantil_Etapa_1_Similac_5HMOs_0_6M_Polvo_1400g.jpg</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/formula-infantil-similac-1-hmo-polvo-1400-gr/COCV_547206.html</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="Q41" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3076,13 +3566,25 @@
       <c r="L42" t="n">
         <v>32</v>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>143</v>
+      </c>
       <c r="N42" t="inlineStr">
         <is>
+          <t>Descubre Similac 2 5HMO: fórmula infantil en polvo de 800g, diseñada para apoyar el desarrollo de tu bebé. Compra ahora y asegura su nutrición.</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw7847c7b6/images/large/545921_3Fomula_Infantil_Etapa_2_Similac_5HMOs_6_12M_Polvo_800g.jpg</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/formula-infantil-similac-2-5hmo-polvo-800-gr/COCV_545921.html</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="Q42" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3139,13 +3641,25 @@
       <c r="L43" t="n">
         <v>33</v>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="n">
+        <v>153</v>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
+          <t>Fórmula Infantil Similac 3 5HMO Polvo 1800 g en Cruz Verde: considera presentación, sabor, formato, etapa y recomendaciones del empaque antes de comprar.</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw890c1655/images/large/547215_4Fomula_Infantil_Etapa_3_Similac_5HMOs_12M_en_Adelante_Polvo_1800g.jpg</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/formula-infantil-similac-3-5hmo-polvo-1800gr/COCV_547215.html</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3202,13 +3716,25 @@
       <c r="L44" t="n">
         <v>32</v>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>240</v>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
+          <t>Similac® 3 Kid es un alimento lácteo en polvo para niños desde los 2 años, con una fórmula científicamente diseñada que incluye grasas de fácil digestión, 5 HMOs (Oligosacáridos), nucleótidos, probiótico, prebióticos, DHA, hierro y luteína.</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw3b2f0b48/images/large/547208_3Fomula_Infantil_Etapa_3_Similac_5HMOs_12M_en_Adelante_Polvo_800g_.jpg</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/similac-3-5-hmos-kid-lata-x-800gr-vainilla/COCV_547208.html</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="Q44" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3265,13 +3791,25 @@
       <c r="L45" t="n">
         <v>32</v>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>240</v>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
+          <t>Similac® 3 Kid es un alimento lácteo en polvo para niños desde los 2 años, con una fórmula científicamente diseñada que incluye grasas de fácil digestión, 5 HMOs (Oligosacáridos), nucleótidos, probiótico, prebióticos, DHA, hierro y luteína.</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw78f6bc87/images/large/546988_3Fomula_Infantil_Etapa_3_Similac_5HMOs_12M_en_Adelante_Polvo_350g.jpg</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/similac-3-5-hmos-kid-lata-x-350gr-vainilla/COCV_546988.html</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="Q45" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3328,13 +3866,25 @@
       <c r="L46" t="n">
         <v>45</v>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>33</v>
+      </c>
       <c r="N46" t="inlineStr">
         <is>
+          <t>Similac Antireflujo Tarro X 375Gr</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dwa0aaf8e6/images/large/113960_3Fomula_Infantil_Especializada_Similac_Anti_Reflujo_0_12M_Polvo_375g.jpg</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/similac-antireflujo-tarro-x-375gr/COCV_113960.html</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="Q46" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3391,13 +3941,25 @@
       <c r="L47" t="n">
         <v>51</v>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="n">
+        <v>38</v>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
+          <t>Similac Neosure Iq Polvo Lata X 370 Gr</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw5cd89b21/images/large/100466_3Fomula_Infantil_Especializada_Similac_NeoSure_Prematuros_0_12M_Polvo_370g.jpg</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/formula-infantil-similac-neosure-polvo-370-gr/COCV_100466.html</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="Q47" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3454,13 +4016,25 @@
       <c r="L48" t="n">
         <v>55</v>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="n">
+        <v>51</v>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
+          <t>Similac Arroz Hmo Lactantes 0-12 Meses Lata X 400Gr</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw58f83df2/images/large/544508_3Fomula_Infantil_Especializada_Similac_Rice_Proteina_de_Arroz_0_36M_Polvo_400g.jpg</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/similac-arroz-hmo-lactantes-0-12-meses-lata-x-400gr/COCV_544508.html</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="Q48" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3517,13 +4091,25 @@
       <c r="L49" t="n">
         <v>54</v>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="n">
+        <v>49</v>
+      </c>
       <c r="N49" t="inlineStr">
         <is>
+          <t>Similac Sensitive Sin Lactosa Polvo Tarro X 400Gr</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw11f08b7d/images/large/96845_3Fomula_Infantil_Especializada_Similac_Sensitive_Sin_Lactosa_0_12M_Polvo_375g_.jpg</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/formula-infantil-similac-sin-lactosa-polvo-375-gr/COCV_96845.html</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="Q49" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
@@ -3580,13 +4166,25 @@
       <c r="L50" t="n">
         <v>41</v>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="n">
+        <v>136</v>
+      </c>
       <c r="N50" t="inlineStr">
         <is>
+          <t>Similac Total Comfort 1 1400 g disponible en Cruz Verde para rutinas de nutrición y bienestar. Compra online y confirma su presentación.</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>https://beta1.cruzverde.com.co/on/demandware.static/-/Sites-masterCatalog_Colombia/default/dw001f8b38/images/large/146187_3Fomula_Infantil_Etapa_1_Similac_Total_Comfort_0_12M_Polvo_1400g.jpg</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
           <t>https://www.cruzverde.com.co/formula-infantil-similac-total-comfort-etapa-1-polvo-1400-gr/COCV_146187.html</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="Q50" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>

</xml_diff>